<commit_message>
Clarify lighthouse visit rewards, overlapping groups and return cooldowns
</commit_message>
<xml_diff>
--- a/docs/arkusze/HARBORLIGHT5-zasady.xlsx
+++ b/docs/arkusze/HARBORLIGHT5-zasady.xlsx
@@ -10931,11 +10931,15 @@
       <c r="A15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>34</v>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Kaplica: płatne błogosławieństwo 100 × poziom, maks. 1/4 h. Latarnia: Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Czlowiek / Blogoslawienstwa. Powrót uruchamia premie i 24 h blokadę osobistą; grupy mają niezależne terminy. Jedyny zgłoszony konflikt: 4 h czy 6 h premii populacji.</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10975,8 +10979,10 @@
       <c r="A19" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>45</v>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Pozostałe szczegóły: bonus pracy podczas przestoju, brakujące pozycje kolejności odejść, moment transakcji portowej i szczegóły Premium. Czas globalnej premii wizyt oczekuje na doprecyzowanie: 4 h czy 6 h.</t>
+        </is>
       </c>
       <c r="C19" s="6" t="s">
         <v>46</v>
@@ -22431,8 +22437,10 @@
       <c r="B18" s="5" t="s">
         <v>922</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>923</v>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania. Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie. Kaplica: płatne błogosławieństwo 100 × poziom, maks. 1/4 h.</t>
+        </is>
       </c>
       <c r="D18" s="5" t="s">
         <v>924</v>
@@ -24145,8 +24153,10 @@
       <c r="C17" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>157</v>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Rozbudowa: 100% szczęścia i produkcja ×2 przez 24 h × nowy poziom. Zwiedzanie: Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
       </c>
       <c r="E17" s="6" t="s">
         <v>158</v>
@@ -24160,8 +24170,10 @@
       <c r="H17" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>161</v>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie. Po zakończeniu premii latarni wracamy do stanu sprzed premii. Zadania latarni są osobną mechaniką z terminem 6 h.</t>
+        </is>
       </c>
       <c r="J17" s="6" t="s">
         <v>93</v>
@@ -24906,17 +24918,23 @@
       <c r="A41" s="6" t="s">
         <v>1252</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>1244</v>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>CZĘŚCIOWO ROZSTRZYGNIĘTE 23.10.2026</t>
+        </is>
       </c>
       <c r="C41" s="6" t="s">
         <v>1253</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>1254</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>1255</v>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Premie startują po powrocie. Osobiste 100% i blokada ponownej wizyty trwają 24 h od powrotu. Odrębne grupy dają sumujące się +10 pp. Pobyt 4 h, bez dojścia i wycofania.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Czas premii populacji: czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Jedna grupa dwóch osób daje +10 pp; dwie odrębne grupy po jednej osobie dają podczas nakładania +20 pp.</t>
+        </is>
       </c>
     </row>
     <row r="42" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29017,14 +29035,20 @@
       <c r="C203" s="6" t="s">
         <v>1927</v>
       </c>
-      <c r="D203" s="6" t="s">
-        <v>1958</v>
-      </c>
-      <c r="E203" s="6" t="s">
-        <v>1992</v>
-      </c>
-      <c r="F203" s="6" t="s">
-        <v>1993</v>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE 23.10.2026</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie.</t>
+        </is>
+      </c>
+      <c r="F203" s="6" t="inlineStr">
+        <is>
+          <t>Źródło: doprecyzowanie użytkownika 23.10.2026. Grupa wysłana o 12:00 wraca do domu o 16:00. Te osoby mogą wyruszyć ponownie najwcześniej o 16:00 następnego dnia.</t>
+        </is>
       </c>
     </row>
     <row r="204" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29037,14 +29061,20 @@
       <c r="C204" s="5" t="s">
         <v>1927</v>
       </c>
-      <c r="D204" s="5" t="s">
-        <v>1996</v>
-      </c>
-      <c r="E204" s="5" t="s">
-        <v>1997</v>
-      </c>
-      <c r="F204" s="5" t="s">
-        <v>1998</v>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE 23.10.2026; CZAS GLOBALNY OTWARTY</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
+      </c>
+      <c r="F204" s="5" t="inlineStr">
+        <is>
+          <t>Źródło: doprecyzowanie użytkownika 23.10.2026. Grupa 2 osób: 12:00 → 16:00. Osobiste 100% i blokada ponownej wizyty do 16:00 następnego dnia; globalnie +10 pp za grupę. Osobne wysłania o 12:00 i 13:00: powroty 16:00 i 17:00; podczas nakładania globalnie +20 pp. Nowy przykład podaje globalny efekt 16:00–20:00, wcześniejsza reguła miała 6 h; pytanie o czas pozostaje otwarte.</t>
+        </is>
       </c>
     </row>
     <row r="205" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29880,11 +29910,15 @@
       <c r="A9" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>2041</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>2042</v>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie. Grupa 2 osób: 12:00 → 16:00. Osobiste 100% i blokada ponownej wizyty do 16:00 następnego dnia; globalnie +10 pp za grupę. Osobne wysłania o 12:00 i 13:00: powroty 16:00 i 17:00; podczas nakładania globalnie +20 pp.</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -30064,8 +30098,10 @@
       <c r="B15" s="6" t="s">
         <v>2069</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>2070</v>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Źródło:701a7d4; oryginał4 zachowany. Pełne wpisy:Twoje wpisy v4. Doprecyzowanie 23.10.2026: pobyt latarni 4 h bez dojścia/wycofania; premie od powrotu; 24 h blokady osobistej; +10 pp na grupę, sumowanie grup. Czas globalnej premii: czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -32790,17 +32826,25 @@
       <c r="A31" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>302</v>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Brak podatku i produkcji, normalne jedzenie.</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie. Grupa 2 osób: 12:00 → 16:00. Osobiste 100% i blokada ponownej wizyty do 16:00 następnego dnia; globalnie +10 pp za grupę. Osobne wysłania o 12:00 i 13:00: powroty 16:00 i 17:00; podczas nakładania globalnie +20 pp.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE 23.10.2026; CZAS GLOBALNEJ PREMII DO DOPRECYZOWANIA</t>
+        </is>
       </c>
     </row>
     <row r="32" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33921,17 +33965,25 @@
       <c r="A27" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>430</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>431</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>432</v>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Pobyt 4 h bez czasu dojścia i możliwości wycofania. Maksymalnie 2 × poziom latarni osób jednocześnie; wysyłamy tylko wolnych mieszkańców z domu. Opłata za samą wizytę nie została ustalona.</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Po powrocie każdy uczestnik otrzymuje 100% szczęścia na 24 h. Jedna wysłana grupa daje całej populacji +10 pp przez czas do doprecyzowania: 4 h w nowym przykładzie, wcześniej 6 h. Premie osobnych grup sumują się przez czas nakładania.</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Ponowne wysłanie konkretnego mieszkańca dopiero 24 h od powrotu. Miejsce zwalnia się po 4 h pobytu i można wysłać inną uprawnioną osobę. Zwiedzający nie produkują, nie płacą podatku i jedzą normalnie. Premia zwiedzania jest odrębna od premii rozbudowy.</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>WIZYTY POTWIERDZONE; CENA NIEOKREŚLONA; CZAS GLOBALNY OTWARTY</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>